<commit_message>
Update dane_pv.xlsx and remove temp files
Delete leftover Office temporary files (~$dane.xlsx and ~$dane_pv.xlsx)
to avoid committing editor artifacts
</commit_message>
<xml_diff>
--- a/dane_pv.xlsx
+++ b/dane_pv.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Użytkownik1\Desktop\python_scripts\animacja_wykresu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5832949-8AC7-4D4E-BFBC-0832CD2DF33B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8481A907-8C22-47B5-9EC0-1DB8BD45A4DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-990" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="102">
   <si>
     <t>Time</t>
   </si>
@@ -337,14 +337,18 @@
   </si>
   <si>
     <t>Moc Pred [W]</t>
+  </si>
+  <si>
+    <t>Cena</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="0.00_ ;[Red]\-0.00\ "/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -355,18 +359,35 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
       <top/>
       <bottom/>
       <diagonal/>
@@ -375,12 +396,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normalny" xfId="0" builtinId="0"/>
@@ -6224,14 +6251,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F99"/>
+  <dimension ref="A1:G99"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.875" customWidth="1"/>
     <col min="2" max="2" width="15.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6247,8 +6274,11 @@
       <c r="F1" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -6269,8 +6299,11 @@
         <f>D2-E2</f>
         <v>30131</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2" s="5">
+        <v>632.04999999999995</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -6291,8 +6324,11 @@
         <f t="shared" ref="F3:F66" si="1">D3-E3</f>
         <v>30357</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G3" s="6">
+        <v>612.28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
@@ -6313,8 +6349,11 @@
         <f t="shared" si="1"/>
         <v>30577</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G4" s="5">
+        <v>565.78</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
@@ -6335,8 +6374,11 @@
         <f t="shared" si="1"/>
         <v>62188</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G5" s="6">
+        <v>632.02</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
@@ -6357,8 +6399,11 @@
         <f t="shared" si="1"/>
         <v>92040</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G6" s="5">
+        <v>634.48</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>7</v>
       </c>
@@ -6379,8 +6424,11 @@
         <f t="shared" si="1"/>
         <v>86533</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G7" s="6">
+        <v>623.75</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>8</v>
       </c>
@@ -6401,8 +6449,11 @@
         <f t="shared" si="1"/>
         <v>80330</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G8" s="5">
+        <v>623.77</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>9</v>
       </c>
@@ -6423,8 +6474,11 @@
         <f t="shared" si="1"/>
         <v>82503</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G9" s="6">
+        <v>623.70000000000005</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>10</v>
       </c>
@@ -6445,8 +6499,11 @@
         <f t="shared" si="1"/>
         <v>92817</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G10" s="5">
+        <v>611.46</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>11</v>
       </c>
@@ -6467,8 +6524,11 @@
         <f t="shared" si="1"/>
         <v>86536</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G11" s="6">
+        <v>609.91</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>12</v>
       </c>
@@ -6489,8 +6549,11 @@
         <f t="shared" si="1"/>
         <v>80551</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G12" s="5">
+        <v>614.38</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>13</v>
       </c>
@@ -6511,8 +6574,11 @@
         <f t="shared" si="1"/>
         <v>83917</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G13" s="6">
+        <v>583.89</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>14</v>
       </c>
@@ -6533,8 +6599,11 @@
         <f t="shared" si="1"/>
         <v>90435</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G14" s="5">
+        <v>568.85</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>15</v>
       </c>
@@ -6555,8 +6624,11 @@
         <f t="shared" si="1"/>
         <v>86265</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G15" s="6">
+        <v>555.58000000000004</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>16</v>
       </c>
@@ -6577,8 +6649,11 @@
         <f t="shared" si="1"/>
         <v>81393</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G16" s="5">
+        <v>519.87</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>17</v>
       </c>
@@ -6599,8 +6674,11 @@
         <f t="shared" si="1"/>
         <v>84344</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G17" s="6">
+        <v>534.64</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>18</v>
       </c>
@@ -6621,8 +6699,11 @@
         <f t="shared" si="1"/>
         <v>88341</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G18" s="5">
+        <v>504.06</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>19</v>
       </c>
@@ -6643,8 +6724,11 @@
         <f t="shared" si="1"/>
         <v>85646</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G19" s="6">
+        <v>514.54</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>20</v>
       </c>
@@ -6665,8 +6749,11 @@
         <f t="shared" si="1"/>
         <v>81528</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G20" s="5">
+        <v>485.29</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>21</v>
       </c>
@@ -6687,8 +6774,11 @@
         <f t="shared" si="1"/>
         <v>87960</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G21" s="6">
+        <v>463.19</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>22</v>
       </c>
@@ -6709,8 +6799,11 @@
         <f t="shared" si="1"/>
         <v>87409</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G22" s="5">
+        <v>1035.17</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>23</v>
       </c>
@@ -6731,8 +6824,11 @@
         <f t="shared" si="1"/>
         <v>94157</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G23" s="6">
+        <v>401.9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>24</v>
       </c>
@@ -6753,8 +6849,11 @@
         <f t="shared" si="1"/>
         <v>86694</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G24" s="5">
+        <v>351.72</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>25</v>
       </c>
@@ -6775,8 +6874,11 @@
         <f t="shared" si="1"/>
         <v>86469</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G25" s="6">
+        <v>253.33</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>26</v>
       </c>
@@ -6797,8 +6899,11 @@
         <f t="shared" si="1"/>
         <v>82495</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G26" s="5">
+        <v>408.76</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>27</v>
       </c>
@@ -6819,8 +6924,11 @@
         <f t="shared" si="1"/>
         <v>84102</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G27" s="6">
+        <v>423.06</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>28</v>
       </c>
@@ -6841,8 +6949,11 @@
         <f t="shared" si="1"/>
         <v>60308</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G28" s="5">
+        <v>382.98</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>29</v>
       </c>
@@ -6863,8 +6974,11 @@
         <f t="shared" si="1"/>
         <v>37757</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G29" s="6">
+        <v>372.07</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>30</v>
       </c>
@@ -6885,8 +6999,11 @@
         <f t="shared" si="1"/>
         <v>13758</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G30" s="5">
+        <v>732.37</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>31</v>
       </c>
@@ -6907,8 +7024,11 @@
         <f t="shared" si="1"/>
         <v>5098</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G31" s="6">
+        <v>412.41</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>32</v>
       </c>
@@ -6929,8 +7049,11 @@
         <f t="shared" si="1"/>
         <v>10694</v>
       </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G32" s="5">
+        <v>408.08</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>33</v>
       </c>
@@ -6951,8 +7074,11 @@
         <f t="shared" si="1"/>
         <v>15591</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G33" s="6">
+        <v>260.02</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>34</v>
       </c>
@@ -6973,8 +7099,11 @@
         <f t="shared" si="1"/>
         <v>-123240</v>
       </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G34" s="5">
+        <v>-4.49</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>35</v>
       </c>
@@ -6995,8 +7124,11 @@
         <f t="shared" si="1"/>
         <v>-45084</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G35" s="6">
+        <v>-31.24</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>36</v>
       </c>
@@ -7017,8 +7149,11 @@
         <f t="shared" si="1"/>
         <v>-29873</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G36" s="5">
+        <v>-780.48</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>37</v>
       </c>
@@ -7039,8 +7174,11 @@
         <f t="shared" si="1"/>
         <v>-46282</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G37" s="6">
+        <v>-39.4</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>38</v>
       </c>
@@ -7061,8 +7199,11 @@
         <f t="shared" si="1"/>
         <v>-61145</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G38" s="5">
+        <v>-104.5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>39</v>
       </c>
@@ -7083,8 +7224,11 @@
         <f t="shared" si="1"/>
         <v>-78996</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G39" s="6">
+        <v>-235.17</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>40</v>
       </c>
@@ -7105,8 +7249,11 @@
         <f t="shared" si="1"/>
         <v>-105179</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G40" s="5">
+        <v>-103.5</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>41</v>
       </c>
@@ -7127,8 +7274,11 @@
         <f t="shared" si="1"/>
         <v>-304351</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G41" s="6">
+        <v>-634.66</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>42</v>
       </c>
@@ -7149,8 +7299,11 @@
         <f t="shared" si="1"/>
         <v>-320389</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G42" s="5">
+        <v>-634.54</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>43</v>
       </c>
@@ -7171,8 +7324,11 @@
         <f t="shared" si="1"/>
         <v>-329193</v>
       </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G43" s="6">
+        <v>-570.71</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>44</v>
       </c>
@@ -7193,8 +7349,11 @@
         <f t="shared" si="1"/>
         <v>-334122</v>
       </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G44" s="5">
+        <v>-564.61</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>45</v>
       </c>
@@ -7215,8 +7374,11 @@
         <f t="shared" si="1"/>
         <v>-345175</v>
       </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G45" s="6">
+        <v>-1516.13</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>46</v>
       </c>
@@ -7237,8 +7399,11 @@
         <f t="shared" si="1"/>
         <v>-348448</v>
       </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G46" s="5">
+        <v>-1511.01</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>47</v>
       </c>
@@ -7259,8 +7424,11 @@
         <f t="shared" si="1"/>
         <v>-355600</v>
       </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G47" s="6">
+        <v>-1519.18</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>48</v>
       </c>
@@ -7281,8 +7449,11 @@
         <f t="shared" si="1"/>
         <v>-354113</v>
       </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G48" s="5">
+        <v>-1529.5</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>49</v>
       </c>
@@ -7303,8 +7474,11 @@
         <f t="shared" si="1"/>
         <v>-364774</v>
       </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G49" s="6">
+        <v>-1539.55</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>50</v>
       </c>
@@ -7325,8 +7499,11 @@
         <f t="shared" si="1"/>
         <v>-369633</v>
       </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G50" s="5">
+        <v>-1596.73</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>51</v>
       </c>
@@ -7347,8 +7524,11 @@
         <f t="shared" si="1"/>
         <v>-375732</v>
       </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G51" s="6">
+        <v>-1603.18</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>52</v>
       </c>
@@ -7369,8 +7549,11 @@
         <f t="shared" si="1"/>
         <v>-363750</v>
       </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G52" s="5">
+        <v>-1619.18</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>53</v>
       </c>
@@ -7391,8 +7574,11 @@
         <f t="shared" si="1"/>
         <v>-365135</v>
       </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G53" s="6">
+        <v>-1603.18</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>54</v>
       </c>
@@ -7413,8 +7599,11 @@
         <f t="shared" si="1"/>
         <v>-362441</v>
       </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G54" s="5">
+        <v>-1179.18</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>55</v>
       </c>
@@ -7435,8 +7624,11 @@
         <f t="shared" si="1"/>
         <v>-359325</v>
       </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G55" s="6">
+        <v>-1179.18</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>56</v>
       </c>
@@ -7457,8 +7649,11 @@
         <f t="shared" si="1"/>
         <v>-344691</v>
       </c>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G56" s="5">
+        <v>-1168.18</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>57</v>
       </c>
@@ -7479,8 +7674,11 @@
         <f t="shared" si="1"/>
         <v>-331416</v>
       </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G57" s="6">
+        <v>-1168.18</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>58</v>
       </c>
@@ -7501,8 +7699,11 @@
         <f t="shared" si="1"/>
         <v>-324799</v>
       </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G58" s="5">
+        <v>-1445.07</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>59</v>
       </c>
@@ -7523,8 +7724,11 @@
         <f t="shared" si="1"/>
         <v>-317873</v>
       </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G59" s="6">
+        <v>-1445.18</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>60</v>
       </c>
@@ -7545,8 +7749,11 @@
         <f t="shared" si="1"/>
         <v>-299397</v>
       </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G60" s="5">
+        <v>-1445.18</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>61</v>
       </c>
@@ -7567,8 +7774,11 @@
         <f t="shared" si="1"/>
         <v>-279566</v>
       </c>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G61" s="6">
+        <v>-1445.09</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>62</v>
       </c>
@@ -7589,8 +7799,11 @@
         <f t="shared" si="1"/>
         <v>-269272</v>
       </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G62" s="5">
+        <v>-1672.18</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>63</v>
       </c>
@@ -7611,8 +7824,11 @@
         <f t="shared" si="1"/>
         <v>-254133</v>
       </c>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G63" s="6">
+        <v>-1672.18</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>64</v>
       </c>
@@ -7633,8 +7849,11 @@
         <f t="shared" si="1"/>
         <v>-239227</v>
       </c>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G64" s="5">
+        <v>-1672.18</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>65</v>
       </c>
@@ -7655,8 +7874,11 @@
         <f t="shared" si="1"/>
         <v>-224375</v>
       </c>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G65" s="6">
+        <v>-1672.18</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>66</v>
       </c>
@@ -7677,8 +7899,11 @@
         <f t="shared" si="1"/>
         <v>-207595</v>
       </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G66" s="5">
+        <v>-2227.1799999999998</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>67</v>
       </c>
@@ -7699,8 +7924,11 @@
         <f t="shared" ref="F67:F99" si="3">D67-E67</f>
         <v>-191728</v>
       </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G67" s="6">
+        <v>-2227.1799999999998</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>68</v>
       </c>
@@ -7721,8 +7949,11 @@
         <f t="shared" si="3"/>
         <v>-166091</v>
       </c>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G68" s="5">
+        <v>-768.56</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>69</v>
       </c>
@@ -7743,8 +7974,11 @@
         <f t="shared" si="3"/>
         <v>-152274</v>
       </c>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G69" s="6">
+        <v>-768.56</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>70</v>
       </c>
@@ -7765,8 +7999,11 @@
         <f t="shared" si="3"/>
         <v>-127193</v>
       </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G70" s="5">
+        <v>-2890.18</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>71</v>
       </c>
@@ -7787,8 +8024,11 @@
         <f t="shared" si="3"/>
         <v>-110409</v>
       </c>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G71" s="6">
+        <v>-2890.18</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>72</v>
       </c>
@@ -7809,8 +8049,11 @@
         <f t="shared" si="3"/>
         <v>-83182</v>
       </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G72" s="5">
+        <v>-17.149999999999999</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>73</v>
       </c>
@@ -7831,8 +8074,11 @@
         <f t="shared" si="3"/>
         <v>-64736</v>
       </c>
-    </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G73" s="6">
+        <v>-33.659999999999997</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
         <v>74</v>
       </c>
@@ -7853,8 +8099,11 @@
         <f t="shared" si="3"/>
         <v>-38107</v>
       </c>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G74" s="5">
+        <v>584.83000000000004</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
         <v>75</v>
       </c>
@@ -7875,8 +8124,11 @@
         <f t="shared" si="3"/>
         <v>-21662</v>
       </c>
-    </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G75" s="6">
+        <v>488.93</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
         <v>76</v>
       </c>
@@ -7897,8 +8149,11 @@
         <f t="shared" si="3"/>
         <v>-18372</v>
       </c>
-    </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G76" s="5">
+        <v>541.29999999999995</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
         <v>77</v>
       </c>
@@ -7919,8 +8174,11 @@
         <f t="shared" si="3"/>
         <v>-12592</v>
       </c>
-    </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G77" s="6">
+        <v>584.03</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
         <v>78</v>
       </c>
@@ -7941,8 +8199,11 @@
         <f t="shared" si="3"/>
         <v>-6479</v>
       </c>
-    </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G78" s="5">
+        <v>623.77</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
         <v>79</v>
       </c>
@@ -7963,8 +8224,11 @@
         <f t="shared" si="3"/>
         <v>1200</v>
       </c>
-    </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G79" s="6">
+        <v>546.65</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
         <v>80</v>
       </c>
@@ -7985,8 +8249,11 @@
         <f t="shared" si="3"/>
         <v>12027</v>
       </c>
-    </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G80" s="5">
+        <v>516.04</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
         <v>81</v>
       </c>
@@ -8007,8 +8274,11 @@
         <f t="shared" si="3"/>
         <v>20768</v>
       </c>
-    </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G81" s="6">
+        <v>597.20000000000005</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
         <v>82</v>
       </c>
@@ -8029,8 +8299,11 @@
         <f t="shared" si="3"/>
         <v>26062</v>
       </c>
-    </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G82" s="5">
+        <v>611.20000000000005</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
         <v>83</v>
       </c>
@@ -8051,8 +8324,11 @@
         <f t="shared" si="3"/>
         <v>29358</v>
       </c>
-    </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G83" s="6">
+        <v>543.98</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
         <v>84</v>
       </c>
@@ -8073,8 +8349,11 @@
         <f t="shared" si="3"/>
         <v>29960</v>
       </c>
-    </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G84" s="5">
+        <v>518.13</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
         <v>85</v>
       </c>
@@ -8095,8 +8374,11 @@
         <f t="shared" si="3"/>
         <v>29515</v>
       </c>
-    </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G85" s="6">
+        <v>454.62</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
         <v>86</v>
       </c>
@@ -8117,8 +8399,11 @@
         <f t="shared" si="3"/>
         <v>29616</v>
       </c>
-    </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G86" s="5">
+        <v>534.07000000000005</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
         <v>87</v>
       </c>
@@ -8139,8 +8424,11 @@
         <f t="shared" si="3"/>
         <v>30077</v>
       </c>
-    </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G87" s="6">
+        <v>619.91999999999996</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
         <v>88</v>
       </c>
@@ -8161,8 +8449,11 @@
         <f t="shared" si="3"/>
         <v>29933</v>
       </c>
-    </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G88" s="5">
+        <v>612.17999999999995</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
         <v>89</v>
       </c>
@@ -8183,8 +8474,11 @@
         <f t="shared" si="3"/>
         <v>29806</v>
       </c>
-    </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G89" s="6">
+        <v>584.01</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
         <v>90</v>
       </c>
@@ -8205,8 +8499,11 @@
         <f t="shared" si="3"/>
         <v>30535</v>
       </c>
-    </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G90" s="5">
+        <v>550.04999999999995</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
         <v>91</v>
       </c>
@@ -8227,8 +8524,11 @@
         <f t="shared" si="3"/>
         <v>29887</v>
       </c>
-    </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G91" s="6">
+        <v>545.99</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
         <v>92</v>
       </c>
@@ -8249,8 +8549,11 @@
         <f t="shared" si="3"/>
         <v>29376</v>
       </c>
-    </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G92" s="5">
+        <v>543.76</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
         <v>93</v>
       </c>
@@ -8271,8 +8574,11 @@
         <f t="shared" si="3"/>
         <v>29817</v>
       </c>
-    </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G93" s="6">
+        <v>525.21</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
         <v>94</v>
       </c>
@@ -8293,8 +8599,11 @@
         <f t="shared" si="3"/>
         <v>30173</v>
       </c>
-    </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G94" s="5">
+        <v>548.85</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
         <v>95</v>
       </c>
@@ -8315,8 +8624,11 @@
         <f t="shared" si="3"/>
         <v>29799</v>
       </c>
-    </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G95" s="6">
+        <v>525.58000000000004</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
         <v>96</v>
       </c>
@@ -8337,8 +8649,11 @@
         <f t="shared" si="3"/>
         <v>29885</v>
       </c>
-    </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G96" s="5">
+        <v>511.33</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97" s="1" t="s">
         <v>97</v>
       </c>
@@ -8359,32 +8674,17 @@
         <f t="shared" si="3"/>
         <v>30218</v>
       </c>
-    </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C98">
-        <v>0</v>
-      </c>
-      <c r="E98" s="4">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="F98" s="4">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C99">
-        <v>0</v>
-      </c>
-      <c r="E99" s="4">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="F99" s="4">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
+      <c r="G97" s="6">
+        <v>507.12</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E98" s="4"/>
+      <c r="F98" s="4"/>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E99" s="4"/>
+      <c r="F99" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>